<commit_message>
plan to remove the IP dashboard and rely on FRED instead
</commit_message>
<xml_diff>
--- a/01_macro_economic/PCE/Z.economic_pulse_monthly/pce_detail.xlsx
+++ b/01_macro_economic/PCE/Z.economic_pulse_monthly/pce_detail.xlsx
@@ -1560,7 +1560,7 @@
         <v>6</v>
       </c>
       <c r="I22" t="n">
-        <v>206310</v>
+        <v>202682</v>
       </c>
       <c r="J22" t="inlineStr">
         <is>
@@ -1568,10 +1568,10 @@
         </is>
       </c>
       <c r="K22" t="n">
-        <v>0.01645062595149072</v>
+        <v>-0.001423848727158061</v>
       </c>
       <c r="L22" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
     </row>
     <row r="23">
@@ -2644,7 +2644,7 @@
         <v>6</v>
       </c>
       <c r="I43" t="n">
-        <v>201130</v>
+        <v>198459</v>
       </c>
       <c r="J43" t="inlineStr">
         <is>
@@ -2652,10 +2652,10 @@
         </is>
       </c>
       <c r="K43" t="n">
-        <v>0.09135403214429116</v>
+        <v>0.07686088532453583</v>
       </c>
       <c r="L43" t="n">
-        <v>80</v>
+        <v>75</v>
       </c>
     </row>
     <row r="44">
@@ -3728,7 +3728,7 @@
         <v>6</v>
       </c>
       <c r="I64" t="n">
-        <v>230667</v>
+        <v>230562</v>
       </c>
       <c r="J64" t="inlineStr">
         <is>
@@ -3736,10 +3736,10 @@
         </is>
       </c>
       <c r="K64" t="n">
-        <v>0.02684787834541202</v>
+        <v>0.02638045549244117</v>
       </c>
       <c r="L64" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="65">
@@ -4812,7 +4812,7 @@
         <v>6</v>
       </c>
       <c r="I85" t="n">
-        <v>87263</v>
+        <v>87273</v>
       </c>
       <c r="J85" t="inlineStr">
         <is>
@@ -4820,10 +4820,10 @@
         </is>
       </c>
       <c r="K85" t="n">
-        <v>0.01683795940245636</v>
+        <v>0.01695448507306163</v>
       </c>
       <c r="L85" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="86">
@@ -5896,7 +5896,7 @@
         <v>6</v>
       </c>
       <c r="I106" t="n">
-        <v>170617</v>
+        <v>168322</v>
       </c>
       <c r="J106" t="inlineStr">
         <is>
@@ -5904,7 +5904,7 @@
         </is>
       </c>
       <c r="K106" t="n">
-        <v>-0.006185963338556255</v>
+        <v>-0.01955393496001256</v>
       </c>
       <c r="L106" t="n">
         <v>3</v>
@@ -6980,7 +6980,7 @@
         <v>6</v>
       </c>
       <c r="I127" t="n">
-        <v>26574</v>
+        <v>26668</v>
       </c>
       <c r="J127" t="inlineStr">
         <is>
@@ -6988,10 +6988,10 @@
         </is>
       </c>
       <c r="K127" t="n">
-        <v>0.0360233918128654</v>
+        <v>0.03968810916179333</v>
       </c>
       <c r="L127" t="n">
-        <v>23</v>
+        <v>30</v>
       </c>
     </row>
     <row r="128">
@@ -8064,7 +8064,7 @@
         <v>6</v>
       </c>
       <c r="I148" t="n">
-        <v>316365</v>
+        <v>315093</v>
       </c>
       <c r="J148" t="inlineStr">
         <is>
@@ -8072,10 +8072,10 @@
         </is>
       </c>
       <c r="K148" t="n">
-        <v>0.03456564037999321</v>
+        <v>0.03040599094164387</v>
       </c>
       <c r="L148" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="149">
@@ -9148,7 +9148,7 @@
         <v>6</v>
       </c>
       <c r="I169" t="n">
-        <v>188941</v>
+        <v>189243</v>
       </c>
       <c r="J169" t="inlineStr">
         <is>
@@ -9156,10 +9156,10 @@
         </is>
       </c>
       <c r="K169" t="n">
-        <v>0.04827452285841094</v>
+        <v>0.04995006657789625</v>
       </c>
       <c r="L169" t="n">
-        <v>45</v>
+        <v>50</v>
       </c>
     </row>
     <row r="170">
@@ -10232,7 +10232,7 @@
         <v>6</v>
       </c>
       <c r="I190" t="n">
-        <v>2217689</v>
+        <v>2215629</v>
       </c>
       <c r="J190" t="inlineStr">
         <is>
@@ -10240,10 +10240,10 @@
         </is>
       </c>
       <c r="K190" t="n">
-        <v>0.04248217002081489</v>
+        <v>0.04151381365062834</v>
       </c>
       <c r="L190" t="n">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="191">
@@ -11316,7 +11316,7 @@
         <v>6</v>
       </c>
       <c r="I211" t="n">
-        <v>8763</v>
+        <v>8743</v>
       </c>
       <c r="J211" t="inlineStr">
         <is>
@@ -11324,10 +11324,10 @@
         </is>
       </c>
       <c r="K211" t="n">
-        <v>0.04321428571428565</v>
+        <v>0.04083333333333328</v>
       </c>
       <c r="L211" t="n">
-        <v>40</v>
+        <v>33</v>
       </c>
     </row>
     <row r="212">
@@ -12400,7 +12400,7 @@
         <v>6</v>
       </c>
       <c r="I232" t="n">
-        <v>268446</v>
+        <v>264718</v>
       </c>
       <c r="J232" t="inlineStr">
         <is>
@@ -12408,10 +12408,10 @@
         </is>
       </c>
       <c r="K232" t="n">
-        <v>0.07667379245895978</v>
+        <v>0.06172166093795739</v>
       </c>
       <c r="L232" t="n">
-        <v>72</v>
+        <v>62</v>
       </c>
     </row>
     <row r="233">
@@ -13484,7 +13484,7 @@
         <v>6</v>
       </c>
       <c r="I253" t="n">
-        <v>340767</v>
+        <v>338685</v>
       </c>
       <c r="J253" t="inlineStr">
         <is>
@@ -13492,10 +13492,10 @@
         </is>
       </c>
       <c r="K253" t="n">
-        <v>0.08555982784819816</v>
+        <v>0.07892733244347894</v>
       </c>
       <c r="L253" t="n">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="254">
@@ -14579,7 +14579,7 @@
         <v>0.04050411597581416</v>
       </c>
       <c r="L274" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="275">
@@ -15663,7 +15663,7 @@
         <v>0.0936739659367396</v>
       </c>
       <c r="L295" t="n">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="296">
@@ -16736,7 +16736,7 @@
         <v>6</v>
       </c>
       <c r="I316" t="n">
-        <v>287624</v>
+        <v>287339</v>
       </c>
       <c r="J316" t="inlineStr">
         <is>
@@ -16744,10 +16744,10 @@
         </is>
       </c>
       <c r="K316" t="n">
-        <v>0.04705912332497264</v>
+        <v>0.04602161654477488</v>
       </c>
       <c r="L316" t="n">
-        <v>43</v>
+        <v>46</v>
       </c>
     </row>
     <row r="317">
@@ -17820,7 +17820,7 @@
         <v>6</v>
       </c>
       <c r="I337" t="n">
-        <v>19771</v>
+        <v>19798</v>
       </c>
       <c r="J337" t="inlineStr">
         <is>
@@ -17828,10 +17828,10 @@
         </is>
       </c>
       <c r="K337" t="n">
-        <v>0.1063174976218455</v>
+        <v>0.1078283252196295</v>
       </c>
       <c r="L337" t="n">
-        <v>86</v>
+        <v>89</v>
       </c>
     </row>
     <row r="338">
@@ -18904,7 +18904,7 @@
         <v>6</v>
       </c>
       <c r="I358" t="n">
-        <v>1112122</v>
+        <v>1103374</v>
       </c>
       <c r="J358" t="inlineStr">
         <is>
@@ -18912,10 +18912,10 @@
         </is>
       </c>
       <c r="K358" t="n">
-        <v>0.1107912720560769</v>
+        <v>0.1020537396199352</v>
       </c>
       <c r="L358" t="n">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="359">
@@ -19988,7 +19988,7 @@
         <v>6</v>
       </c>
       <c r="I379" t="n">
-        <v>36308</v>
+        <v>36311</v>
       </c>
       <c r="J379" t="inlineStr">
         <is>
@@ -19996,10 +19996,10 @@
         </is>
       </c>
       <c r="K379" t="n">
-        <v>0.07077975698950101</v>
+        <v>0.07086823168573786</v>
       </c>
       <c r="L379" t="n">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="380">
@@ -21072,7 +21072,7 @@
         <v>6</v>
       </c>
       <c r="I400" t="n">
-        <v>1253215</v>
+        <v>1261782</v>
       </c>
       <c r="J400" t="inlineStr">
         <is>
@@ -21080,10 +21080,10 @@
         </is>
       </c>
       <c r="K400" t="n">
-        <v>0.03880984254742437</v>
+        <v>0.04591116508274662</v>
       </c>
       <c r="L400" t="n">
-        <v>29</v>
+        <v>45</v>
       </c>
     </row>
     <row r="401">
@@ -22156,7 +22156,7 @@
         <v>6</v>
       </c>
       <c r="I421" t="n">
-        <v>285801</v>
+        <v>286455</v>
       </c>
       <c r="J421" t="inlineStr">
         <is>
@@ -22164,10 +22164,10 @@
         </is>
       </c>
       <c r="K421" t="n">
-        <v>0.09372392943247476</v>
+        <v>0.0962267039148903</v>
       </c>
       <c r="L421" t="n">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="422">
@@ -23240,7 +23240,7 @@
         <v>6</v>
       </c>
       <c r="I442" t="n">
-        <v>29372</v>
+        <v>29710</v>
       </c>
       <c r="J442" t="inlineStr">
         <is>
@@ -23248,10 +23248,10 @@
         </is>
       </c>
       <c r="K442" t="n">
-        <v>0.1119439712284687</v>
+        <v>0.1247397312133258</v>
       </c>
       <c r="L442" t="n">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
     <row r="443">
@@ -24324,7 +24324,7 @@
         <v>6</v>
       </c>
       <c r="I463" t="n">
-        <v>219622</v>
+        <v>218334</v>
       </c>
       <c r="J463" t="inlineStr">
         <is>
@@ -24332,10 +24332,10 @@
         </is>
       </c>
       <c r="K463" t="n">
-        <v>0.1065306986164714</v>
+        <v>0.1000413144026038</v>
       </c>
       <c r="L463" t="n">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="464">
@@ -25408,7 +25408,7 @@
         <v>6</v>
       </c>
       <c r="I484" t="n">
-        <v>415527</v>
+        <v>415949</v>
       </c>
       <c r="J484" t="inlineStr">
         <is>
@@ -25416,7 +25416,7 @@
         </is>
       </c>
       <c r="K484" t="n">
-        <v>0.03695875143804739</v>
+        <v>0.03801186373425636</v>
       </c>
       <c r="L484" t="n">
         <v>25</v>
@@ -26492,7 +26492,7 @@
         <v>6</v>
       </c>
       <c r="I505" t="n">
-        <v>6398507</v>
+        <v>6391334</v>
       </c>
       <c r="J505" t="inlineStr">
         <is>
@@ -26500,10 +26500,10 @@
         </is>
       </c>
       <c r="K505" t="n">
-        <v>0.04060188796217568</v>
+        <v>0.03943532874103983</v>
       </c>
       <c r="L505" t="n">
-        <v>34</v>
+        <v>28</v>
       </c>
     </row>
     <row r="506">
@@ -27576,7 +27576,7 @@
         <v>6</v>
       </c>
       <c r="I526" t="n">
-        <v>72321</v>
+        <v>73967</v>
       </c>
       <c r="J526" t="inlineStr">
         <is>
@@ -27584,7 +27584,7 @@
         </is>
       </c>
       <c r="K526" t="n">
-        <v>0.1198668318364819</v>
+        <v>0.1453545989470424</v>
       </c>
       <c r="L526" t="n">
         <v>92</v>
@@ -28660,7 +28660,7 @@
         <v>6</v>
       </c>
       <c r="I547" t="n">
-        <v>101435</v>
+        <v>101424</v>
       </c>
       <c r="J547" t="inlineStr">
         <is>
@@ -28668,7 +28668,7 @@
         </is>
       </c>
       <c r="K547" t="n">
-        <v>0.1139848005622914</v>
+        <v>0.1138639957828149</v>
       </c>
       <c r="L547" t="n">
         <v>90</v>
@@ -29755,7 +29755,7 @@
         <v>0.05009276437847876</v>
       </c>
       <c r="L568" t="n">
-        <v>46</v>
+        <v>51</v>
       </c>
     </row>
     <row r="569">
@@ -30828,7 +30828,7 @@
         <v>6</v>
       </c>
       <c r="I589" t="n">
-        <v>207853</v>
+        <v>207806</v>
       </c>
       <c r="J589" t="inlineStr">
         <is>
@@ -30836,10 +30836,10 @@
         </is>
       </c>
       <c r="K589" t="n">
-        <v>0.01350178463458884</v>
+        <v>0.01327261024750825</v>
       </c>
       <c r="L589" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="590">
@@ -31912,7 +31912,7 @@
         <v>6</v>
       </c>
       <c r="I610" t="n">
-        <v>119699</v>
+        <v>119481</v>
       </c>
       <c r="J610" t="inlineStr">
         <is>
@@ -31920,10 +31920,10 @@
         </is>
       </c>
       <c r="K610" t="n">
-        <v>0.04634736924919358</v>
+        <v>0.04444172487040743</v>
       </c>
       <c r="L610" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="611">
@@ -32996,7 +32996,7 @@
         <v>6</v>
       </c>
       <c r="I631" t="n">
-        <v>275679</v>
+        <v>275636</v>
       </c>
       <c r="J631" t="inlineStr">
         <is>
@@ -33004,10 +33004,10 @@
         </is>
       </c>
       <c r="K631" t="n">
-        <v>0.03751053772505575</v>
+        <v>0.03734870837598603</v>
       </c>
       <c r="L631" t="n">
-        <v>27</v>
+        <v>24</v>
       </c>
     </row>
     <row r="632">
@@ -34080,7 +34080,7 @@
         <v>6</v>
       </c>
       <c r="I652" t="n">
-        <v>195498</v>
+        <v>194936</v>
       </c>
       <c r="J652" t="inlineStr">
         <is>
@@ -34088,10 +34088,10 @@
         </is>
       </c>
       <c r="K652" t="n">
-        <v>0.03983873026679707</v>
+        <v>0.03684949576613761</v>
       </c>
       <c r="L652" t="n">
-        <v>31</v>
+        <v>23</v>
       </c>
     </row>
     <row r="653">
@@ -35164,7 +35164,7 @@
         <v>6</v>
       </c>
       <c r="I673" t="n">
-        <v>1814778</v>
+        <v>1819583</v>
       </c>
       <c r="J673" t="inlineStr">
         <is>
@@ -35172,10 +35172,10 @@
         </is>
       </c>
       <c r="K673" t="n">
-        <v>0.05895327606700396</v>
+        <v>0.06175707382711693</v>
       </c>
       <c r="L673" t="n">
-        <v>57</v>
+        <v>63</v>
       </c>
     </row>
     <row r="674">
@@ -36248,7 +36248,7 @@
         <v>6</v>
       </c>
       <c r="I694" t="n">
-        <v>3207133</v>
+        <v>3207163</v>
       </c>
       <c r="J694" t="inlineStr">
         <is>
@@ -36256,10 +36256,10 @@
         </is>
       </c>
       <c r="K694" t="n">
-        <v>0.05766770692178036</v>
+        <v>0.05767760050312165</v>
       </c>
       <c r="L694" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="695">
@@ -37332,7 +37332,7 @@
         <v>6</v>
       </c>
       <c r="I715" t="n">
-        <v>1552000</v>
+        <v>1557991</v>
       </c>
       <c r="J715" t="inlineStr">
         <is>
@@ -37340,10 +37340,10 @@
         </is>
       </c>
       <c r="K715" t="n">
-        <v>0.05536447474537298</v>
+        <v>0.05943837201869728</v>
       </c>
       <c r="L715" t="n">
-        <v>52</v>
+        <v>59</v>
       </c>
     </row>
     <row r="716">
@@ -38416,7 +38416,7 @@
         <v>6</v>
       </c>
       <c r="I736" t="n">
-        <v>601576</v>
+        <v>592340</v>
       </c>
       <c r="J736" t="inlineStr">
         <is>
@@ -38424,10 +38424,10 @@
         </is>
       </c>
       <c r="K736" t="n">
-        <v>0.117124478184006</v>
+        <v>0.09997325925155609</v>
       </c>
       <c r="L736" t="n">
-        <v>91</v>
+        <v>85</v>
       </c>
     </row>
     <row r="737">
@@ -39500,7 +39500,7 @@
         <v>6</v>
       </c>
       <c r="I757" t="n">
-        <v>538826</v>
+        <v>538439</v>
       </c>
       <c r="J757" t="inlineStr">
         <is>
@@ -39508,10 +39508,10 @@
         </is>
       </c>
       <c r="K757" t="n">
-        <v>0.04578484422672324</v>
+        <v>0.04503373211499206</v>
       </c>
       <c r="L757" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
     <row r="758">
@@ -40584,7 +40584,7 @@
         <v>6</v>
       </c>
       <c r="I778" t="n">
-        <v>117141</v>
+        <v>114358</v>
       </c>
       <c r="J778" t="inlineStr">
         <is>
@@ -40592,10 +40592,10 @@
         </is>
       </c>
       <c r="K778" t="n">
-        <v>0.07536881144944974</v>
+        <v>0.04982052859149366</v>
       </c>
       <c r="L778" t="n">
-        <v>71</v>
+        <v>49</v>
       </c>
     </row>
     <row r="779">
@@ -41668,7 +41668,7 @@
         <v>6</v>
       </c>
       <c r="I799" t="n">
-        <v>101821</v>
+        <v>101857</v>
       </c>
       <c r="J799" t="inlineStr">
         <is>
@@ -41676,10 +41676,10 @@
         </is>
       </c>
       <c r="K799" t="n">
-        <v>-0.001098760950820621</v>
+        <v>-0.0007455877880568895</v>
       </c>
       <c r="L799" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="800">
@@ -42752,7 +42752,7 @@
         <v>6</v>
       </c>
       <c r="I820" t="n">
-        <v>130397</v>
+        <v>130258</v>
       </c>
       <c r="J820" t="inlineStr">
         <is>
@@ -42760,10 +42760,10 @@
         </is>
       </c>
       <c r="K820" t="n">
-        <v>0.03513507077025668</v>
+        <v>0.03403164220336419</v>
       </c>
       <c r="L820" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="821">
@@ -43836,7 +43836,7 @@
         <v>6</v>
       </c>
       <c r="I841" t="n">
-        <v>47029</v>
+        <v>47536</v>
       </c>
       <c r="J841" t="inlineStr">
         <is>
@@ -43844,10 +43844,10 @@
         </is>
       </c>
       <c r="K841" t="n">
-        <v>0.03120203481997974</v>
+        <v>0.04231899311494103</v>
       </c>
       <c r="L841" t="n">
-        <v>20</v>
+        <v>38</v>
       </c>
     </row>
     <row r="842">
@@ -44920,7 +44920,7 @@
         <v>6</v>
       </c>
       <c r="I862" t="n">
-        <v>145756</v>
+        <v>145200</v>
       </c>
       <c r="J862" t="inlineStr">
         <is>
@@ -44928,10 +44928,10 @@
         </is>
       </c>
       <c r="K862" t="n">
-        <v>0.03683364395566868</v>
+        <v>0.03287854429569359</v>
       </c>
       <c r="L862" t="n">
-        <v>24</v>
+        <v>20</v>
       </c>
     </row>
     <row r="863">
@@ -46004,7 +46004,7 @@
         <v>6</v>
       </c>
       <c r="I883" t="n">
-        <v>406956</v>
+        <v>406553</v>
       </c>
       <c r="J883" t="inlineStr">
         <is>
@@ -46012,7 +46012,7 @@
         </is>
       </c>
       <c r="K883" t="n">
-        <v>-0.02371642013040909</v>
+        <v>-0.02468321330384171</v>
       </c>
       <c r="L883" t="n">
         <v>2</v>
@@ -47088,7 +47088,7 @@
         <v>6</v>
       </c>
       <c r="I904" t="n">
-        <v>8542</v>
+        <v>8520</v>
       </c>
       <c r="J904" t="inlineStr">
         <is>
@@ -47096,10 +47096,10 @@
         </is>
       </c>
       <c r="K904" t="n">
-        <v>0.0001170823088632034</v>
+        <v>-0.002458728486125716</v>
       </c>
       <c r="L904" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="905">
@@ -48172,7 +48172,7 @@
         <v>6</v>
       </c>
       <c r="I925" t="n">
-        <v>129847</v>
+        <v>129042</v>
       </c>
       <c r="J925" t="inlineStr">
         <is>
@@ -48180,10 +48180,10 @@
         </is>
       </c>
       <c r="K925" t="n">
-        <v>0.04210239083153433</v>
+        <v>0.03564176852513223</v>
       </c>
       <c r="L925" t="n">
-        <v>37</v>
+        <v>22</v>
       </c>
     </row>
     <row r="926">
@@ -49256,7 +49256,7 @@
         <v>6</v>
       </c>
       <c r="I946" t="n">
-        <v>380693</v>
+        <v>381638</v>
       </c>
       <c r="J946" t="inlineStr">
         <is>
@@ -49264,10 +49264,10 @@
         </is>
       </c>
       <c r="K946" t="n">
-        <v>0.06984018142934634</v>
+        <v>0.07249586191585577</v>
       </c>
       <c r="L946" t="n">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
     <row r="947">
@@ -50340,7 +50340,7 @@
         <v>6</v>
       </c>
       <c r="I967" t="n">
-        <v>4180819</v>
+        <v>4175706</v>
       </c>
       <c r="J967" t="inlineStr">
         <is>
@@ -50348,10 +50348,10 @@
         </is>
       </c>
       <c r="K967" t="n">
-        <v>0.0396075032027563</v>
+        <v>0.03833609844596686</v>
       </c>
       <c r="L967" t="n">
-        <v>30</v>
+        <v>26</v>
       </c>
     </row>
     <row r="968">
@@ -51424,7 +51424,7 @@
         <v>6</v>
       </c>
       <c r="I988" t="n">
-        <v>65605</v>
+        <v>65743</v>
       </c>
       <c r="J988" t="inlineStr">
         <is>
@@ -51432,10 +51432,10 @@
         </is>
       </c>
       <c r="K988" t="n">
-        <v>0.06944331241339952</v>
+        <v>0.07169288450566458</v>
       </c>
       <c r="L988" t="n">
-        <v>65</v>
+        <v>70</v>
       </c>
     </row>
     <row r="989">
@@ -52508,7 +52508,7 @@
         <v>6</v>
       </c>
       <c r="I1009" t="n">
-        <v>122205</v>
+        <v>122048</v>
       </c>
       <c r="J1009" t="inlineStr">
         <is>
@@ -52516,7 +52516,7 @@
         </is>
       </c>
       <c r="K1009" t="n">
-        <v>0.05073772183243919</v>
+        <v>0.0493878112532673</v>
       </c>
       <c r="L1009" t="n">
         <v>48</v>
@@ -53592,7 +53592,7 @@
         <v>6</v>
       </c>
       <c r="I1030" t="n">
-        <v>405585</v>
+        <v>406241</v>
       </c>
       <c r="J1030" t="inlineStr">
         <is>
@@ -53600,10 +53600,10 @@
         </is>
       </c>
       <c r="K1030" t="n">
-        <v>0.06476790036596181</v>
+        <v>0.06649007387494299</v>
       </c>
       <c r="L1030" t="n">
-        <v>63</v>
+        <v>66</v>
       </c>
     </row>
     <row r="1031">
@@ -54676,7 +54676,7 @@
         <v>6</v>
       </c>
       <c r="I1051" t="n">
-        <v>214872</v>
+        <v>214861</v>
       </c>
       <c r="J1051" t="inlineStr">
         <is>
@@ -54684,10 +54684,10 @@
         </is>
       </c>
       <c r="K1051" t="n">
-        <v>0.04124325817378294</v>
+        <v>0.04118995352804067</v>
       </c>
       <c r="L1051" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="1052">
@@ -55760,7 +55760,7 @@
         <v>6</v>
       </c>
       <c r="I1072" t="n">
-        <v>262778</v>
+        <v>261591</v>
       </c>
       <c r="J1072" t="inlineStr">
         <is>
@@ -55768,10 +55768,10 @@
         </is>
       </c>
       <c r="K1072" t="n">
-        <v>0.08065716694425595</v>
+        <v>0.07577570785269261</v>
       </c>
       <c r="L1072" t="n">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="1073">
@@ -56844,7 +56844,7 @@
         <v>6</v>
       </c>
       <c r="I1093" t="n">
-        <v>118217</v>
+        <v>117887</v>
       </c>
       <c r="J1093" t="inlineStr">
         <is>
@@ -56852,10 +56852,10 @@
         </is>
       </c>
       <c r="K1093" t="n">
-        <v>0.01420715333602152</v>
+        <v>0.01137601770746643</v>
       </c>
       <c r="L1093" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="1094">
@@ -57928,7 +57928,7 @@
         <v>6</v>
       </c>
       <c r="I1114" t="n">
-        <v>510546</v>
+        <v>511034</v>
       </c>
       <c r="J1114" t="inlineStr">
         <is>
@@ -57936,10 +57936,10 @@
         </is>
       </c>
       <c r="K1114" t="n">
-        <v>0.1034204031173951</v>
+        <v>0.104475095851686</v>
       </c>
       <c r="L1114" t="n">
-        <v>85</v>
+        <v>88</v>
       </c>
     </row>
     <row r="1115">
@@ -59012,7 +59012,7 @@
         <v>6</v>
       </c>
       <c r="I1135" t="n">
-        <v>209141</v>
+        <v>208109</v>
       </c>
       <c r="J1135" t="inlineStr">
         <is>
@@ -59020,10 +59020,10 @@
         </is>
       </c>
       <c r="K1135" t="n">
-        <v>0.05010493969733187</v>
+        <v>0.04492322832668894</v>
       </c>
       <c r="L1135" t="n">
-        <v>47</v>
+        <v>42</v>
       </c>
     </row>
     <row r="1136">
@@ -60096,7 +60096,7 @@
         <v>6</v>
       </c>
       <c r="I1156" t="n">
-        <v>111635</v>
+        <v>111957</v>
       </c>
       <c r="J1156" t="inlineStr">
         <is>
@@ -60104,10 +60104,10 @@
         </is>
       </c>
       <c r="K1156" t="n">
-        <v>0.05675934077376721</v>
+        <v>0.05980745747309224</v>
       </c>
       <c r="L1156" t="n">
-        <v>54</v>
+        <v>60</v>
       </c>
     </row>
     <row r="1157">
@@ -61180,7 +61180,7 @@
         <v>6</v>
       </c>
       <c r="I1177" t="n">
-        <v>1633604</v>
+        <v>1629440</v>
       </c>
       <c r="J1177" t="inlineStr">
         <is>
@@ -61188,10 +61188,10 @@
         </is>
       </c>
       <c r="K1177" t="n">
-        <v>0.07486393161313409</v>
+        <v>0.07212414068997464</v>
       </c>
       <c r="L1177" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="1178">
@@ -62264,7 +62264,7 @@
         <v>6</v>
       </c>
       <c r="I1198" t="n">
-        <v>108735</v>
+        <v>109681</v>
       </c>
       <c r="J1198" t="inlineStr">
         <is>
@@ -62272,10 +62272,10 @@
         </is>
       </c>
       <c r="K1198" t="n">
-        <v>0.01703238116617101</v>
+        <v>0.02588061432553257</v>
       </c>
       <c r="L1198" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="1199">
@@ -63348,7 +63348,7 @@
         <v>6</v>
       </c>
       <c r="I1219" t="n">
-        <v>2437502</v>
+        <v>2437525</v>
       </c>
       <c r="J1219" t="inlineStr">
         <is>
@@ -63356,10 +63356,10 @@
         </is>
       </c>
       <c r="K1219" t="n">
-        <v>0.05993924324531164</v>
+        <v>0.05994924471509289</v>
       </c>
       <c r="L1219" t="n">
-        <v>59</v>
+        <v>61</v>
       </c>
     </row>
     <row r="1220">
@@ -64432,7 +64432,7 @@
         <v>6</v>
       </c>
       <c r="I1240" t="n">
-        <v>20526289</v>
+        <v>20493341</v>
       </c>
       <c r="J1240" t="inlineStr">
         <is>
@@ -64440,10 +64440,10 @@
         </is>
       </c>
       <c r="K1240" t="n">
-        <v>0.05670665425983046</v>
+        <v>0.05501046987674241</v>
       </c>
       <c r="L1240" t="n">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="1241">
@@ -65516,7 +65516,7 @@
         <v>6</v>
       </c>
       <c r="I1261" t="n">
-        <v>239675</v>
+        <v>239904</v>
       </c>
       <c r="J1261" t="inlineStr">
         <is>
@@ -65524,10 +65524,10 @@
         </is>
       </c>
       <c r="K1261" t="n">
-        <v>0.05290556687987635</v>
+        <v>0.05391157657974266</v>
       </c>
       <c r="L1261" t="n">
-        <v>50</v>
+        <v>55</v>
       </c>
     </row>
     <row r="1262">
@@ -66600,7 +66600,7 @@
         <v>6</v>
       </c>
       <c r="I1282" t="n">
-        <v>703480</v>
+        <v>709057</v>
       </c>
       <c r="J1282" t="inlineStr">
         <is>
@@ -66608,10 +66608,10 @@
         </is>
       </c>
       <c r="K1282" t="n">
-        <v>0.07763150235446581</v>
+        <v>0.08617467470994278</v>
       </c>
       <c r="L1282" t="n">
-        <v>73</v>
+        <v>80</v>
       </c>
     </row>
     <row r="1283">
@@ -67684,7 +67684,7 @@
         <v>6</v>
       </c>
       <c r="I1303" t="n">
-        <v>820285</v>
+        <v>818568</v>
       </c>
       <c r="J1303" t="inlineStr">
         <is>
@@ -67692,7 +67692,7 @@
         </is>
       </c>
       <c r="K1303" t="n">
-        <v>0.07126392648981272</v>
+        <v>0.06902158369214728</v>
       </c>
       <c r="L1303" t="n">
         <v>68</v>
@@ -68768,7 +68768,7 @@
         <v>6</v>
       </c>
       <c r="I1324" t="n">
-        <v>1216907</v>
+        <v>1225471</v>
       </c>
       <c r="J1324" t="inlineStr">
         <is>
@@ -68776,10 +68776,10 @@
         </is>
       </c>
       <c r="K1324" t="n">
-        <v>0.03788528145727832</v>
+        <v>0.04518941361396767</v>
       </c>
       <c r="L1324" t="n">
-        <v>28</v>
+        <v>44</v>
       </c>
     </row>
     <row r="1325">
@@ -69852,7 +69852,7 @@
         <v>6</v>
       </c>
       <c r="I1345" t="n">
-        <v>624378</v>
+        <v>621628</v>
       </c>
       <c r="J1345" t="inlineStr">
         <is>
@@ -69860,10 +69860,10 @@
         </is>
       </c>
       <c r="K1345" t="n">
-        <v>0.08801865240552242</v>
+        <v>0.08322660128566373</v>
       </c>
       <c r="L1345" t="n">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="1346">
@@ -70936,7 +70936,7 @@
         <v>6</v>
       </c>
       <c r="I1366" t="n">
-        <v>287241</v>
+        <v>283731</v>
       </c>
       <c r="J1366" t="inlineStr">
         <is>
@@ -70944,10 +70944,10 @@
         </is>
       </c>
       <c r="K1366" t="n">
-        <v>0.06355224621126565</v>
+        <v>0.05055595256167678</v>
       </c>
       <c r="L1366" t="n">
-        <v>61</v>
+        <v>53</v>
       </c>
     </row>
     <row r="1367">
@@ -72020,7 +72020,7 @@
         <v>6</v>
       </c>
       <c r="I1387" t="n">
-        <v>17019</v>
+        <v>17222</v>
       </c>
       <c r="J1387" t="inlineStr">
         <is>
@@ -72028,10 +72028,10 @@
         </is>
       </c>
       <c r="K1387" t="n">
-        <v>-0.00111515436084042</v>
+        <v>0.01079938959971827</v>
       </c>
       <c r="L1387" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="1388">
@@ -73104,7 +73104,7 @@
         <v>6</v>
       </c>
       <c r="I1408" t="n">
-        <v>309450</v>
+        <v>306767</v>
       </c>
       <c r="J1408" t="inlineStr">
         <is>
@@ -73112,10 +73112,10 @@
         </is>
       </c>
       <c r="K1408" t="n">
-        <v>0.09840377386618959</v>
+        <v>0.08888037000358495</v>
       </c>
       <c r="L1408" t="n">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="1409">
@@ -74188,7 +74188,7 @@
         <v>6</v>
       </c>
       <c r="I1429" t="n">
-        <v>32044</v>
+        <v>31898</v>
       </c>
       <c r="J1429" t="inlineStr">
         <is>
@@ -74196,10 +74196,10 @@
         </is>
       </c>
       <c r="K1429" t="n">
-        <v>0.05508544335056476</v>
+        <v>0.05027822593921827</v>
       </c>
       <c r="L1429" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="1430">
@@ -75272,7 +75272,7 @@
         <v>6</v>
       </c>
       <c r="I1450" t="n">
-        <v>329942</v>
+        <v>326481</v>
       </c>
       <c r="J1450" t="inlineStr">
         <is>
@@ -75280,10 +75280,10 @@
         </is>
       </c>
       <c r="K1450" t="n">
-        <v>0.06009889569684845</v>
+        <v>0.04897875252620998</v>
       </c>
       <c r="L1450" t="n">
-        <v>60</v>
+        <v>47</v>
       </c>
     </row>
     <row r="1451">
@@ -76356,7 +76356,7 @@
         <v>6</v>
       </c>
       <c r="I1471" t="n">
-        <v>319954</v>
+        <v>316645</v>
       </c>
       <c r="J1471" t="inlineStr">
         <is>
@@ -76364,10 +76364,10 @@
         </is>
       </c>
       <c r="K1471" t="n">
-        <v>0.09079813583071106</v>
+        <v>0.07951697969119165</v>
       </c>
       <c r="L1471" t="n">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
     <row r="1472">
@@ -77440,7 +77440,7 @@
         <v>6</v>
       </c>
       <c r="I1492" t="n">
-        <v>14127781</v>
+        <v>14102007</v>
       </c>
       <c r="J1492" t="inlineStr">
         <is>
@@ -77448,10 +77448,10 @@
         </is>
       </c>
       <c r="K1492" t="n">
-        <v>0.06416571293504125</v>
+        <v>0.06222430351730002</v>
       </c>
       <c r="L1492" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="1493">
@@ -78524,7 +78524,7 @@
         <v>6</v>
       </c>
       <c r="I1513" t="n">
-        <v>348376</v>
+        <v>348170</v>
       </c>
       <c r="J1513" t="inlineStr">
         <is>
@@ -78532,7 +78532,7 @@
         </is>
       </c>
       <c r="K1513" t="n">
-        <v>0.05947971218120673</v>
+        <v>0.05885322579664121</v>
       </c>
       <c r="L1513" t="n">
         <v>58</v>
@@ -79608,7 +79608,7 @@
         <v>6</v>
       </c>
       <c r="I1534" t="n">
-        <v>124317</v>
+        <v>123755</v>
       </c>
       <c r="J1534" t="inlineStr">
         <is>
@@ -79616,10 +79616,10 @@
         </is>
       </c>
       <c r="K1534" t="n">
-        <v>0.02605645427533831</v>
+        <v>0.02141795972268068</v>
       </c>
       <c r="L1534" t="n">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="1535">
@@ -80692,7 +80692,7 @@
         <v>6</v>
       </c>
       <c r="I1555" t="n">
-        <v>97212</v>
+        <v>98767</v>
       </c>
       <c r="J1555" t="inlineStr">
         <is>
@@ -80700,10 +80700,10 @@
         </is>
       </c>
       <c r="K1555" t="n">
-        <v>0.02567024340835</v>
+        <v>0.04207683136559792</v>
       </c>
       <c r="L1555" t="n">
-        <v>16</v>
+        <v>37</v>
       </c>
     </row>
     <row r="1556">
@@ -81776,7 +81776,7 @@
         <v>6</v>
       </c>
       <c r="I1576" t="n">
-        <v>35306</v>
+        <v>35385</v>
       </c>
       <c r="J1576" t="inlineStr">
         <is>
@@ -81784,10 +81784,10 @@
         </is>
       </c>
       <c r="K1576" t="n">
-        <v>0.01635097011917774</v>
+        <v>0.01862513673786625</v>
       </c>
       <c r="L1576" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="1577">
@@ -82860,7 +82860,7 @@
         <v>6</v>
       </c>
       <c r="I1597" t="n">
-        <v>182204</v>
+        <v>183513</v>
       </c>
       <c r="J1597" t="inlineStr">
         <is>
@@ -82868,10 +82868,10 @@
         </is>
       </c>
       <c r="K1597" t="n">
-        <v>0.01322389420884629</v>
+        <v>0.02050315304794625</v>
       </c>
       <c r="L1597" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
     </row>
     <row r="1598">
@@ -83944,7 +83944,7 @@
         <v>6</v>
       </c>
       <c r="I1618" t="n">
-        <v>357910</v>
+        <v>357914</v>
       </c>
       <c r="J1618" t="inlineStr">
         <is>
@@ -83952,10 +83952,10 @@
         </is>
       </c>
       <c r="K1618" t="n">
-        <v>0.0298234760966205</v>
+        <v>0.02983498539757434</v>
       </c>
       <c r="L1618" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="1619">
@@ -85028,7 +85028,7 @@
         <v>6</v>
       </c>
       <c r="I1639" t="n">
-        <v>737669</v>
+        <v>737676</v>
       </c>
       <c r="J1639" t="inlineStr">
         <is>
@@ -85036,10 +85036,10 @@
         </is>
       </c>
       <c r="K1639" t="n">
-        <v>0.05093329990112805</v>
+        <v>0.05094327257599884</v>
       </c>
       <c r="L1639" t="n">
-        <v>49</v>
+        <v>54</v>
       </c>
     </row>
     <row r="1640">
@@ -86112,7 +86112,7 @@
         <v>6</v>
       </c>
       <c r="I1660" t="n">
-        <v>1292633</v>
+        <v>1287264</v>
       </c>
       <c r="J1660" t="inlineStr">
         <is>
@@ -86120,10 +86120,10 @@
         </is>
       </c>
       <c r="K1660" t="n">
-        <v>0.04295567027111646</v>
+        <v>0.03862371449272795</v>
       </c>
       <c r="L1660" t="n">
-        <v>39</v>
+        <v>27</v>
       </c>
     </row>
     <row r="1661">
@@ -87196,7 +87196,7 @@
         <v>6</v>
       </c>
       <c r="I1681" t="n">
-        <v>112978</v>
+        <v>112748</v>
       </c>
       <c r="J1681" t="inlineStr">
         <is>
@@ -87204,10 +87204,10 @@
         </is>
       </c>
       <c r="K1681" t="n">
-        <v>0.06904741628107236</v>
+        <v>0.06687105534580473</v>
       </c>
       <c r="L1681" t="n">
-        <v>64</v>
+        <v>67</v>
       </c>
     </row>
     <row r="1682">
@@ -89364,7 +89364,7 @@
         <v>6</v>
       </c>
       <c r="I1723" t="n">
-        <v>60874</v>
+        <v>61096</v>
       </c>
       <c r="J1723" t="inlineStr">
         <is>
@@ -89372,7 +89372,7 @@
         </is>
       </c>
       <c r="K1723" t="n">
-        <v>0.02038284890542763</v>
+        <v>0.02410405980756991</v>
       </c>
       <c r="L1723" t="n">
         <v>15</v>
@@ -90448,7 +90448,7 @@
         <v>6</v>
       </c>
       <c r="I1744" t="n">
-        <v>60439</v>
+        <v>60389</v>
       </c>
       <c r="J1744" t="inlineStr">
         <is>
@@ -90456,10 +90456,10 @@
         </is>
       </c>
       <c r="K1744" t="n">
-        <v>0.04034770634305884</v>
+        <v>0.03948704707806172</v>
       </c>
       <c r="L1744" t="n">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
     <row r="1745">
@@ -91532,7 +91532,7 @@
         <v>6</v>
       </c>
       <c r="I1765" t="n">
-        <v>484284</v>
+        <v>481063</v>
       </c>
       <c r="J1765" t="inlineStr">
         <is>
@@ -91540,10 +91540,10 @@
         </is>
       </c>
       <c r="K1765" t="n">
-        <v>0.08226176269459229</v>
+        <v>0.07506357911297634</v>
       </c>
       <c r="L1765" t="n">
-        <v>76</v>
+        <v>73</v>
       </c>
     </row>
     <row r="1766">
@@ -92616,7 +92616,7 @@
         <v>6</v>
       </c>
       <c r="I1786" t="n">
-        <v>415957</v>
+        <v>414163</v>
       </c>
       <c r="J1786" t="inlineStr">
         <is>
@@ -92624,10 +92624,10 @@
         </is>
       </c>
       <c r="K1786" t="n">
-        <v>0.04798820891385946</v>
+        <v>0.04346829256002627</v>
       </c>
       <c r="L1786" t="n">
-        <v>44</v>
+        <v>40</v>
       </c>
     </row>
     <row r="1787">
@@ -93700,7 +93700,7 @@
         <v>6</v>
       </c>
       <c r="I1807" t="n">
-        <v>84451</v>
+        <v>84365</v>
       </c>
       <c r="J1807" t="inlineStr">
         <is>
@@ -93708,10 +93708,10 @@
         </is>
       </c>
       <c r="K1807" t="n">
-        <v>0.04111396025445035</v>
+        <v>0.0400537501849203</v>
       </c>
       <c r="L1807" t="n">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="1808">
@@ -94795,7 +94795,7 @@
         <v>0.09252110056361906</v>
       </c>
       <c r="L1828" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="1829">
@@ -95879,7 +95879,7 @@
         <v>0.0796612827348282</v>
       </c>
       <c r="L1849" t="n">
-        <v>74</v>
+        <v>78</v>
       </c>
     </row>
     <row r="1850">
@@ -96952,7 +96952,7 @@
         <v>6</v>
       </c>
       <c r="I1870" t="n">
-        <v>243197</v>
+        <v>244081</v>
       </c>
       <c r="J1870" t="inlineStr">
         <is>
@@ -96960,10 +96960,10 @@
         </is>
       </c>
       <c r="K1870" t="n">
-        <v>0.0371360703487158</v>
+        <v>0.04090597000285734</v>
       </c>
       <c r="L1870" t="n">
-        <v>26</v>
+        <v>34</v>
       </c>
     </row>
     <row r="1871">
@@ -98036,7 +98036,7 @@
         <v>6</v>
       </c>
       <c r="I1891" t="n">
-        <v>100193</v>
+        <v>98765</v>
       </c>
       <c r="J1891" t="inlineStr">
         <is>
@@ -98044,10 +98044,10 @@
         </is>
       </c>
       <c r="K1891" t="n">
-        <v>0.05761334248165939</v>
+        <v>0.04253971605003426</v>
       </c>
       <c r="L1891" t="n">
-        <v>55</v>
+        <v>39</v>
       </c>
     </row>
     <row r="1892">
@@ -99120,7 +99120,7 @@
         <v>6</v>
       </c>
       <c r="I1912" t="n">
-        <v>143516</v>
+        <v>142378</v>
       </c>
       <c r="J1912" t="inlineStr">
         <is>
@@ -99128,10 +99128,10 @@
         </is>
       </c>
       <c r="K1912" t="n">
-        <v>0.07450305094897614</v>
+        <v>0.0659828547898027</v>
       </c>
       <c r="L1912" t="n">
-        <v>69</v>
+        <v>65</v>
       </c>
     </row>
     <row r="1913">
@@ -99761,7 +99761,7 @@
         <v>0</v>
       </c>
       <c r="L1933" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>